<commit_message>
Improve phone number processing and data cleaning for customer imports
Refactor `process-excel.js` to extract only digits for phone numbers, handling international formats and ensuring accurate storage in `processed-customers.json`.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: 3a403264-fd9e-4adc-a1fe-abb166e7fc2e
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/d1299512-b679-4553-b6bf-6043a19b76b9/3a403264-fd9e-4adc-a1fe-abb166e7fc2e/Uyesc4J
</commit_message>
<xml_diff>
--- a/clientes_procesados.xlsx
+++ b/clientes_procesados.xlsx
@@ -564,7 +564,7 @@
         <v>S/ La Altagracia C/ Juan Jose D</v>
       </c>
       <c r="D12" t="str">
-        <v>18092400364y8299094181</v>
+        <v>18092400364</v>
       </c>
     </row>
     <row r="13">
@@ -592,7 +592,7 @@
         <v>S/ Las Colinas C/Simon Bolivar #7</v>
       </c>
       <c r="D14" t="str">
-        <v>18292345062/8092494428</v>
+        <v>18292345062</v>
       </c>
     </row>
     <row r="15">
@@ -690,7 +690,7 @@
         <v>C/ Inmaculada C S/ Santa Fé Casa# #20</v>
       </c>
       <c r="D21" t="str">
-        <v>1N/A</v>
+        <v/>
       </c>
     </row>
     <row r="22">
@@ -1082,7 +1082,7 @@
         <v>las colinas, al lado de. Prof. Wilfrido</v>
       </c>
       <c r="D49" t="str">
-        <v>18092237569/8095852049</v>
+        <v>18092237569</v>
       </c>
     </row>
     <row r="50">
@@ -1096,7 +1096,7 @@
         <v>Anacaona 16, (encima de jose luis)</v>
       </c>
       <c r="D50" t="str">
-        <v>18295363512/8096102751</v>
+        <v>18295363512</v>
       </c>
     </row>
     <row r="51">
@@ -1922,7 +1922,7 @@
         <v>la estancia al lado de adalgiza</v>
       </c>
       <c r="D109" t="str">
-        <v>184940495444</v>
+        <v>18494049544</v>
       </c>
     </row>
     <row r="110">
@@ -2790,7 +2790,7 @@
         <v>santa fe. Casa crema con azul</v>
       </c>
       <c r="D171" t="str">
-        <v>18097091002/8097161003</v>
+        <v>18097091002</v>
       </c>
     </row>
     <row r="172">

</xml_diff>